<commit_message>
feat: implement e2e test suite and test cases for project import functionality
</commit_message>
<xml_diff>
--- a/test_plan.xlsx
+++ b/test_plan.xlsx
@@ -451,7 +451,7 @@
         <v>-</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as document staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Open Import Project page</v>
       </c>
       <c r="G2" t="str">
@@ -487,7 +487,7 @@
         <v>-</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as representative_x000d_
+        <v xml:space="preserve">1. Login as user `facilities_rep` with password `facilities_rep` (Role: Facilities Rep)_x000d_
 2. Open Import Project page</v>
       </c>
       <c r="G3" t="str">
@@ -523,7 +523,7 @@
         <v>Import Project URL: /app/project-import</v>
       </c>
       <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as guest_x000d_
+        <v xml:space="preserve">1. Login as user `guest` with password `guest` (Role: Guest)_x000d_
 2. Open Import Project URL</v>
       </c>
       <c r="G4" t="str">
@@ -559,7 +559,7 @@
         <v>Import Project URL: /app/project-import</v>
       </c>
       <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as finance staff_x000d_
+        <v xml:space="preserve">1. Login as user `finance_staff` with password `finance_staff` (Role: Finance Staff)_x000d_
 2. Open import URL</v>
       </c>
       <c r="G5" t="str">
@@ -595,7 +595,7 @@
         <v>Import Project URL: /app/project-import</v>
       </c>
       <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as contract staff_x000d_
+        <v xml:space="preserve">1. Login as user `contract` with password `contract` (Role: Contract)_x000d_
 2. Open import URL</v>
       </c>
       <c r="G6" t="str">
@@ -631,7 +631,7 @@
         <v>Import Project URL: /app/project-import</v>
       </c>
       <c r="F7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as procurement staff_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Open import URL</v>
       </c>
       <c r="G7" t="str">
@@ -667,7 +667,7 @@
         <v>Import Project URL: /app/project-import</v>
       </c>
       <c r="F8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as procurement head_x000d_
+        <v xml:space="preserve">1. Login as user `proc_head1` with password `proc_head1` (Role: Procurement Head1)_x000d_
 2. Open import URL</v>
       </c>
       <c r="G8" t="str">
@@ -707,7 +707,7 @@
         <v>Upload non-.xlsx/.xls file to the system</v>
       </c>
       <c r="G9" t="str">
-        <v>Error says only Excel files are supported</v>
+        <v>UI shows error: "รองรับเฉพาะไฟล์ Excel .xlsx และ .xls"</v>
       </c>
       <c r="H9" t="str">
         <v>P1</v>
@@ -743,7 +743,7 @@
         <v>Upload .xlsx/.xls file over 50 rows to the system</v>
       </c>
       <c r="G10" t="str">
-        <v>Error says file must not exceed 50 rows</v>
+        <v>UI shows error indicating the file must not exceed 50 rows (Note: Exact message depends on implementation, e.g., "จำนวนแถวต้องไม่เกิน 50 แถว")</v>
       </c>
       <c r="H10" t="str">
         <v>P1</v>
@@ -848,7 +848,7 @@
         <v>LessPaper Excel file containing row with `lesspaper_no` = 9999</v>
       </c>
       <c r="F13" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Click the submit button</v>
@@ -886,7 +886,7 @@
         <v>LessPaper Excel file containing 2 rows with the same `lesspaper_no` = 8888</v>
       </c>
       <c r="F14" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Click the submit button</v>
@@ -927,7 +927,7 @@
 - Row 3: `budget` = -500</v>
       </c>
       <c r="F15" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Click the submit button</v>
@@ -967,7 +967,7 @@
         <v>LessPaper Excel file with procurement method "LT100K" but `budget` = 150000</v>
       </c>
       <c r="F16" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Click the submit button</v>
@@ -1005,7 +1005,7 @@
         <v>LessPaper Excel file with past delivery date</v>
       </c>
       <c r="F17" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Click the submit button</v>
@@ -1043,7 +1043,7 @@
         <v>LessPaper Excel file with valid rows</v>
       </c>
       <c r="F18" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Edit an editable cell (e.g., Budget) in the data table</v>
@@ -1081,7 +1081,7 @@
         <v>LessPaper Excel file with 2 valid rows</v>
       </c>
       <c r="F19" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the LessPaper Excel file_x000d_
 4. Click the delete icon (ลบ) on the first row</v>
@@ -1119,7 +1119,7 @@
         <v>Fiori Excel file with a missing PR Number (`pr_no` is empty)</v>
       </c>
       <c r="F20" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Click the submit button</v>
@@ -1158,7 +1158,7 @@
         <v>Fiori Excel file containing `pr_no` = "1000000001"</v>
       </c>
       <c r="F21" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Click the submit button</v>
@@ -1196,7 +1196,7 @@
         <v>Fiori Excel file with 2 rows having duplicate `pr_no` = "1000000002"</v>
       </c>
       <c r="F22" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Click the submit button</v>
@@ -1234,7 +1234,7 @@
         <v>Fiori Excel file without specifying the procurement method</v>
       </c>
       <c r="F23" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file</v>
       </c>
@@ -1273,7 +1273,7 @@
 - Row 2: `budget` = -100</v>
       </c>
       <c r="F24" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Click the submit button</v>
@@ -1313,7 +1313,7 @@
         <v>Fiori Excel file with method "LT500K" but `budget` = 600000</v>
       </c>
       <c r="F25" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Click the submit button</v>
@@ -1351,7 +1351,7 @@
         <v>Fiori Excel file with past delivery date</v>
       </c>
       <c r="F26" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Click the submit button</v>
@@ -1389,7 +1389,7 @@
         <v>Fiori Excel file with 2 valid rows</v>
       </c>
       <c r="F27" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Upload the Fiori Excel file_x000d_
 4. Edit a cell (e.g., Budget) on the first row_x000d_
@@ -1429,7 +1429,7 @@
         <v>-</v>
       </c>
       <c r="F28" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Unit Representative_x000d_
+        <v xml:space="preserve">1. Login as user `facilities_rep` with password `facilities_rep` (Role: Facilities Rep)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>-</v>
       </c>
       <c r="F29" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Unit Representative_x000d_
+        <v xml:space="preserve">1. Login as user `facilities_rep` with password `facilities_rep` (Role: Facilities Rep)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form</v>
       </c>
@@ -1503,7 +1503,7 @@
         <v>-</v>
       </c>
       <c r="F30" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>-</v>
       </c>
       <c r="F31" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Leave required fields empty and click the submit button ("ยืนยัน")</v>
@@ -1579,7 +1579,7 @@
         <v>Form data with `pr_no` = "1000000001"</v>
       </c>
       <c r="F32" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Fill in the existing PR number_x000d_
@@ -1618,7 +1618,7 @@
         <v>Form data with budget as "abc", "0", or "-100"</v>
       </c>
       <c r="F33" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Enter non-number, 0, or negative value in the budget field_x000d_
@@ -1657,7 +1657,7 @@
         <v>Form data with procurement method "LT100K" but budget set to 150000</v>
       </c>
       <c r="F34" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Select method "LT100K" and enter budget 150000_x000d_
@@ -1697,7 +1697,7 @@
         <v>Select a specific unit and fiscal year that have available budget plans</v>
       </c>
       <c r="F35" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Select the specific unit and fiscal year_x000d_
@@ -1737,7 +1737,7 @@
         <v>-</v>
       </c>
       <c r="F36" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Select unit and fiscal year_x000d_
@@ -1777,7 +1777,7 @@
         <v>Select 2 budget plans with amounts 10,000 and 20,000</v>
       </c>
       <c r="F37" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Select multiple budget plans from the dropdown</v>
@@ -1815,7 +1815,7 @@
         <v>Select budget plans summing to 30,000, then override the budget field to 20,000</v>
       </c>
       <c r="F38" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Select budget plans_x000d_
@@ -1855,7 +1855,7 @@
         <v>Select a delivery date that is earlier than the standard working-day threshold (e.g., 2 days from now)</v>
       </c>
       <c r="F39" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Open manual creation form_x000d_
 4. Select an early delivery date_x000d_
@@ -1894,7 +1894,7 @@
         <v>Select fiscal year "2568"</v>
       </c>
       <c r="F40" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Create a project using either manual form or import, specifying fiscal year 2568_x000d_
 4. Check the generated receive number</v>
@@ -1932,7 +1932,7 @@
         <v>Dates across different urgency thresholds</v>
       </c>
       <c r="F41" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Create projects with delivery dates crossing different urgency thresholds_x000d_
 4. Inspect the API payload or database</v>
@@ -1970,7 +1970,7 @@
         <v>Valid manual form data</v>
       </c>
       <c r="F42" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Fill and submit the manual creation form successfully_x000d_
 4. Check the project status</v>
@@ -2008,7 +2008,7 @@
         <v>Project with specific procurement method</v>
       </c>
       <c r="F43" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Create a project with a specific procurement method_x000d_
 4. Check the workgroup pools</v>
@@ -2046,7 +2046,7 @@
         <v>Valid manual form data</v>
       </c>
       <c r="F44" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Unit Representative_x000d_
+        <v xml:space="preserve">1. Login as user `facilities_rep` with password `facilities_rep` (Role: Facilities Rep)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Create a project successfully_x000d_
 4. Click "create more" or equivalent success action button</v>
@@ -2122,7 +2122,7 @@
         <v>Valid manual form data</v>
       </c>
       <c r="F46" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Create a project successfully_x000d_
 4. Click "back to all projects" action button</v>
@@ -2160,7 +2160,7 @@
         <v>-</v>
       </c>
       <c r="F47" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Click the LessPaper template download button</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>-</v>
       </c>
       <c r="F48" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Document Staff_x000d_
+        <v xml:space="preserve">1. Login as user `document_staff` with password `document_staff` (Role: Document Staff)_x000d_
 2. Navigate to Import Project Page_x000d_
 3. Click the Fiori template download button</v>
       </c>

</xml_diff>

<commit_message>
test: implement end-to-end test suite for project listing, filtering, and search functionality
</commit_message>
<xml_diff>
--- a/test_plan.xlsx
+++ b/test_plan.xlsx
@@ -2463,7 +2463,7 @@
         <v>-</v>
       </c>
       <c r="F55" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Staff_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page</v>
       </c>
       <c r="G55" t="str">
@@ -2605,7 +2605,7 @@
         <v>-</v>
       </c>
       <c r="F59" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Staff_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page</v>
       </c>
       <c r="G59" t="str">
@@ -2965,7 +2965,7 @@
         <v>-</v>
       </c>
       <c r="F69" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Staff_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Expand the status filter options</v>
       </c>
@@ -3002,7 +3002,7 @@
         <v>-</v>
       </c>
       <c r="F70" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as External Staff_x000d_
+        <v xml:space="preserve">1. Login as user `registration_staff` with password `registration_staff` (Role: Guest)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Apply status filters</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>-</v>
       </c>
       <c r="F73" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Staff_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Open advanced filters</v>
       </c>
@@ -3150,7 +3150,7 @@
         <v>-</v>
       </c>
       <c r="F74" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as External Staff_x000d_
+        <v xml:space="preserve">1. Login as user `registration_staff` with password `registration_staff` (Role: Guest)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Open advanced filters</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>1. User is authorized and logged in</v>
       </c>
       <c r="E77" t="str">
-        <v>Projects exist in various statuses</v>
+        <v>Observe rows in the table matching statuses like "รอการตอบรับ", "ยังไม่ได้มอบหมาย", "รออนุมัติยกเลิก", etc.</v>
       </c>
       <c r="F77" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3293,7 +3293,7 @@
         <v>1. User is authorized and logged in</v>
       </c>
       <c r="E78" t="str">
-        <v>Project is currently in the procurement phase</v>
+        <v>Project: "User Testing - Network monitoring sensors"</v>
       </c>
       <c r="F78" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3329,7 +3329,7 @@
         <v>1. User is authorized and logged in</v>
       </c>
       <c r="E79" t="str">
-        <v>Project is currently in the contract phase</v>
+        <v>Project: "User Testing - Security service contract"</v>
       </c>
       <c r="F79" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3365,10 +3365,10 @@
         <v>1. User is authorized as the original assignee of a project</v>
       </c>
       <c r="E80" t="str">
-        <v>Target project is in `IN_PROGRESS` status</v>
+        <v>Project: "User Testing - Network monitoring sensors" (Status: IN_PROGRESS)</v>
       </c>
       <c r="F80" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as the Original Assignee_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Click the three dots menu on the target project</v>
       </c>
@@ -3402,10 +3402,10 @@
         <v>1. User is authorized as the Procurement Head</v>
       </c>
       <c r="E81" t="str">
-        <v>Target project is in `IN_PROGRESS` status</v>
+        <v>Project: "User Testing - Network monitoring sensors" (Status: IN_PROGRESS)</v>
       </c>
       <c r="F81" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as the Procurement Head_x000d_
+        <v xml:space="preserve">1. Login as user `proc_head1` with password `proc_head1` (Role: Procurement Head1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Click the three dots menu on the target project</v>
       </c>
@@ -3439,10 +3439,10 @@
         <v>1. User is authorized as Admin</v>
       </c>
       <c r="E82" t="str">
-        <v>Target project is in `IN_PROGRESS` status</v>
+        <v>Project: "User Testing - Network monitoring sensors" (Status: IN_PROGRESS)</v>
       </c>
       <c r="F82" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Admin_x000d_
+        <v xml:space="preserve">1. Login as user `super_admin` with password `super_admin` (Role: Super Admin)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Click the three dots menu on the target project</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>1. User is authorized as an eligible assignee</v>
       </c>
       <c r="E84" t="str">
-        <v>Projects in UNASSIGNED, WAITING_ACCEPT, CLOSED, CANCELLED, WAITING_CANCEL, and REQUEST_EDIT statuses</v>
+        <v>Projects like "User Testing - New chairs for reading room", "User Testing - Completed tablet procurement"</v>
       </c>
       <c r="F84" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3549,10 +3549,10 @@
         <v>1. User is authorized as the Original Assignee</v>
       </c>
       <c r="E85" t="str">
-        <v>Target project is at step 1 and has no uploaded files or data</v>
+        <v>Project: "User Testing - Network monitoring sensors"</v>
       </c>
       <c r="F85" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Original Assignee_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Click the three dots menu and select the return action_x000d_
 4. Confirm the return</v>
@@ -3587,10 +3587,10 @@
         <v>1. User is authorized as an added Assignee or the Workgroup Head</v>
       </c>
       <c r="E86" t="str">
-        <v>Target project is at step 1 and has no uploaded files or data</v>
+        <v>Project: "User Testing - Network monitoring sensors"</v>
       </c>
       <c r="F86" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Added Assignee or Procurement Head_x000d_
+        <v xml:space="preserve">1. Login as user `procurement2` with password `procurement2` (Role: Procurement2) or Procurement Head_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Click the three dots menu on the target project</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>1. User is authorized as the Original Assignee</v>
       </c>
       <c r="E87" t="str">
-        <v>Target project has moved past step 1, or has data/uploaded docs</v>
+        <v>Project: "User Testing - Accounting software renewal"</v>
       </c>
       <c r="F87" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3660,7 +3660,7 @@
         <v>1. User is authorized</v>
       </c>
       <c r="E88" t="str">
-        <v>Projects in CLOSED, CANCELLED, WAITING_CANCEL, and REQUEST_EDIT statuses</v>
+        <v>Projects like "User Testing - Completed tablet procurement", "User Testing - Cancelled printer repair"</v>
       </c>
       <c r="F88" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3696,7 +3696,7 @@
         <v>1. User is authorized</v>
       </c>
       <c r="E89" t="str">
-        <v>Eligible project for cancellation</v>
+        <v>Project: "User Testing - Data center UPS upgrade"</v>
       </c>
       <c r="F89" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to All Projects Page_x000d_
@@ -3733,10 +3733,10 @@
         <v>1. User is authorized as Procurement Staff</v>
       </c>
       <c r="E90" t="str">
-        <v>Eligible project and valid reason</v>
+        <v>Project: "User Testing - Data center UPS upgrade" with reason "Duplicate plan"</v>
       </c>
       <c r="F90" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Staff_x000d_
+        <v xml:space="preserve">1. Login as user `procurement1` with password `procurement1` (Role: Procurement1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Open cancel dialog for a project_x000d_
 4. Enter a reason and submit</v>
@@ -3771,10 +3771,10 @@
         <v>1. User is authorized as Procurement Head</v>
       </c>
       <c r="E91" t="str">
-        <v>Eligible project and valid reason</v>
+        <v>Project: "User Testing - Data center UPS upgrade" with reason "Duplicate plan"</v>
       </c>
       <c r="F91" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Head_x000d_
+        <v xml:space="preserve">1. Login as user `proc_head1` with password `proc_head1` (Role: Procurement Head1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Open cancel dialog for a project_x000d_
 4. Enter a reason and submit</v>
@@ -3809,10 +3809,10 @@
         <v>1. User is authorized as Procurement Head</v>
       </c>
       <c r="E92" t="str">
-        <v>Project in WAITING_CANCEL status</v>
+        <v>Project: "User Testing - Air purifier order"</v>
       </c>
       <c r="F92" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login as Procurement Head_x000d_
+        <v xml:space="preserve">1. Login as user `proc_head1` with password `proc_head1` (Role: Procurement Head1)_x000d_
 2. Navigate to All Projects Page_x000d_
 3. Approve or Reject the WAITING_CANCEL request</v>
       </c>

</xml_diff>